<commit_message>
docs: documents 26/05/10 work
</commit_message>
<xml_diff>
--- a/doc/基本設計/00_勤怠管理システム_設計書.xlsx
+++ b/doc/基本設計/00_勤怠管理システム_設計書.xlsx
@@ -5,16 +5,16 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="TOP" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="00_メイン" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="01_画面一覧" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="02_画面遷移図" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="03_機能一覧" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="04_API一覧" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="05_テーブル定義" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="03_API一覧" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="04_テーブル定義" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="05_機能一覧" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -37,22 +37,22 @@
     <t xml:space="preserve">一覧</t>
   </si>
   <si>
-    <t xml:space="preserve">01_メイン</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02_画面一覧</t>
-  </si>
-  <si>
-    <t xml:space="preserve">03_画面遷移図</t>
-  </si>
-  <si>
-    <t xml:space="preserve">04_機能一覧</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05_API一覧</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06_テーブル定義</t>
+    <t xml:space="preserve">00_メイン</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01_画面一覧</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02_画面遷移図</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_API一覧</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04_テーブル定義</t>
+  </si>
+  <si>
+    <t xml:space="preserve">05_機能一覧</t>
   </si>
   <si>
     <t xml:space="preserve">■ドキュメント一覧</t>
@@ -266,6 +266,174 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">■API一覧</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ログイン</t>
+  </si>
+  <si>
+    <t xml:space="preserve">email,password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">token</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/attendance/clock-in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">出勤登録</t>
+  </si>
+  <si>
+    <t xml:space="preserve">userId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">success</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/attendance/clock-out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">退勤登録</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">勤怠一覧取得</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attendanceList</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/attendance/summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">月次集計取得</t>
+  </si>
+  <si>
+    <t xml:space="preserve">summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">■テーブル定義</t>
+  </si>
+  <si>
+    <t xml:space="preserve">usersテーブル</t>
+  </si>
+  <si>
+    <t xml:space="preserve">カラム名</t>
+  </si>
+  <si>
+    <t xml:space="preserve">型</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NULL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bigint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">○</t>
+  </si>
+  <si>
+    <t xml:space="preserve">×</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ユーザーID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">varchar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">名前</t>
+  </si>
+  <si>
+    <t xml:space="preserve">email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">メール</t>
+  </si>
+  <si>
+    <t xml:space="preserve">password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">パスワード</t>
+  </si>
+  <si>
+    <t xml:space="preserve">role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attendancesテーブル</t>
+  </si>
+  <si>
+    <t xml:space="preserve">勤怠ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">user_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">work_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">勤務日</t>
+  </si>
+  <si>
+    <t xml:space="preserve">clock_in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">datetime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">出勤</t>
+  </si>
+  <si>
+    <t xml:space="preserve">clock_out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">退勤</t>
+  </si>
+  <si>
     <t xml:space="preserve">■機能一覧</t>
   </si>
   <si>
@@ -278,9 +446,6 @@
     <t xml:space="preserve">FUNC-001</t>
   </si>
   <si>
-    <t xml:space="preserve">ログイン</t>
-  </si>
-  <si>
     <t xml:space="preserve">ユーザー認証</t>
   </si>
   <si>
@@ -290,18 +455,12 @@
     <t xml:space="preserve">出勤打刻</t>
   </si>
   <si>
-    <t xml:space="preserve">出勤登録</t>
-  </si>
-  <si>
     <t xml:space="preserve">FUNC-003</t>
   </si>
   <si>
     <t xml:space="preserve">退勤打刻</t>
   </si>
   <si>
-    <t xml:space="preserve">退勤登録</t>
-  </si>
-  <si>
     <t xml:space="preserve">FUNC-004</t>
   </si>
   <si>
@@ -327,165 +486,6 @@
   </si>
   <si>
     <t xml:space="preserve">社員管理</t>
-  </si>
-  <si>
-    <t xml:space="preserve">■API一覧</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Method</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Request</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Response</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POST</t>
-  </si>
-  <si>
-    <t xml:space="preserve">email,password</t>
-  </si>
-  <si>
-    <t xml:space="preserve">token</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/attendance/clock-in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">userId</t>
-  </si>
-  <si>
-    <t xml:space="preserve">success</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API-003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/attendance/clock-out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API-004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">勤怠一覧取得</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attendanceList</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API-005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/attendance/summary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">月次集計取得</t>
-  </si>
-  <si>
-    <t xml:space="preserve">summary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">■テーブル定義</t>
-  </si>
-  <si>
-    <t xml:space="preserve">usersテーブル</t>
-  </si>
-  <si>
-    <t xml:space="preserve">カラム名</t>
-  </si>
-  <si>
-    <t xml:space="preserve">型</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NULL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bigint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">○</t>
-  </si>
-  <si>
-    <t xml:space="preserve">×</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ユーザーID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">varchar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">名前</t>
-  </si>
-  <si>
-    <t xml:space="preserve">email</t>
-  </si>
-  <si>
-    <t xml:space="preserve">メール</t>
-  </si>
-  <si>
-    <t xml:space="preserve">password</t>
-  </si>
-  <si>
-    <t xml:space="preserve">パスワード</t>
-  </si>
-  <si>
-    <t xml:space="preserve">role</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attendancesテーブル</t>
-  </si>
-  <si>
-    <t xml:space="preserve">勤怠ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">user_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">work_date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">勤務日</t>
-  </si>
-  <si>
-    <t xml:space="preserve">clock_in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">datetime</t>
-  </si>
-  <si>
-    <t xml:space="preserve">出勤</t>
-  </si>
-  <si>
-    <t xml:space="preserve">clock_out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">退勤</t>
   </si>
 </sst>
 </file>
@@ -935,9 +935,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>674640</xdr:colOff>
+      <xdr:colOff>674280</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>10440</xdr:rowOff>
+      <xdr:rowOff>10080</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -947,7 +947,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="282960" y="1698840"/>
-          <a:ext cx="1525320" cy="577440"/>
+          <a:ext cx="1524960" cy="577080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1008,9 +1008,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>674640</xdr:colOff>
+      <xdr:colOff>674280</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>99720</xdr:rowOff>
+      <xdr:rowOff>99360</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1020,7 +1020,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="282960" y="736560"/>
-          <a:ext cx="1525320" cy="577440"/>
+          <a:ext cx="1524960" cy="577080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1081,9 +1081,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>137520</xdr:colOff>
+      <xdr:colOff>137160</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>103320</xdr:rowOff>
+      <xdr:rowOff>102960</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1093,7 +1093,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2184120" y="2492640"/>
-          <a:ext cx="1525320" cy="577440"/>
+          <a:ext cx="1524960" cy="577080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1154,9 +1154,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>161640</xdr:colOff>
+      <xdr:colOff>161280</xdr:colOff>
       <xdr:row>29</xdr:row>
-      <xdr:rowOff>146880</xdr:rowOff>
+      <xdr:rowOff>146520</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1166,7 +1166,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2208240" y="4563000"/>
-          <a:ext cx="1525320" cy="577440"/>
+          <a:ext cx="1524960" cy="577080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1227,9 +1227,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>137520</xdr:colOff>
+      <xdr:colOff>137160</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>27720</xdr:rowOff>
+      <xdr:rowOff>27360</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1239,7 +1239,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2184120" y="3456000"/>
-          <a:ext cx="1525320" cy="577440"/>
+          <a:ext cx="1524960" cy="577080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1300,9 +1300,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>173160</xdr:colOff>
+      <xdr:colOff>172800</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>14040</xdr:rowOff>
+      <xdr:rowOff>13680</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1312,7 +1312,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2219760" y="5580720"/>
-          <a:ext cx="1525320" cy="577440"/>
+          <a:ext cx="1524960" cy="577080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2038,26 +2038,21 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:F11"/>
+  <dimension ref="B1:G10"/>
   <sheetFormatPr defaultColWidth="10.4921875" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.6"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F2" s="10"/>
-    </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="F3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
@@ -2067,87 +2062,117 @@
         <v>62</v>
       </c>
       <c r="D5" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="3"/>
+      <c r="F5" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="8" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="E6" s="8"/>
-      <c r="F6" s="3"/>
+        <v>32</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>67</v>
-      </c>
       <c r="D7" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="E7" s="8"/>
-      <c r="F7" s="3"/>
+        <v>71</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="E8" s="8"/>
-      <c r="F8" s="3"/>
+        <v>76</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="8" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="C9" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="E9" s="8"/>
+      <c r="G9" s="8" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="E10" s="8"/>
-    </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="E11" s="8"/>
+        <v>83</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>85</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2165,140 +2190,218 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:G10"/>
-  <sheetFormatPr defaultColWidth="10.4921875" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="B1:F19"/>
+  <sheetFormatPr defaultColWidth="10.4921875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.81"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.85"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="5" t="s">
-        <v>81</v>
-      </c>
-    </row>
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="6" t="s">
+      <c r="B5" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>12</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="8" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>68</v>
+        <v>95</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="D8" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>71</v>
-      </c>
       <c r="F8" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="8" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>42</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="D9" s="4"/>
       <c r="E9" s="8" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>101</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="D10" s="4"/>
       <c r="E10" s="8" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="F10" s="8" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="13" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="G10" s="8" t="s">
-        <v>103</v>
+      <c r="C15" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" s="4"/>
+      <c r="E16" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D18" s="4"/>
+      <c r="E18" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -2317,219 +2420,116 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:F19"/>
-  <sheetFormatPr defaultColWidth="10.4921875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="B1:F11"/>
+  <sheetFormatPr defaultColWidth="10.4921875" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.42"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F2" s="10"/>
+    </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="5" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+        <v>116</v>
+      </c>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F4" s="3"/>
+    </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="13" t="s">
-        <v>105</v>
-      </c>
+      <c r="B5" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>12</v>
-      </c>
+      <c r="B6" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="E6" s="8"/>
+      <c r="F6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="8" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>114</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="E7" s="8"/>
+      <c r="F7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>117</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="E8" s="8"/>
+      <c r="F8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="8" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>119</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="E9" s="8"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>121</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="E10" s="8"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="13" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="D16" s="4"/>
-      <c r="E16" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="D17" s="4"/>
-      <c r="E17" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="D18" s="4"/>
-      <c r="E18" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="C19" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="F19" s="8" t="s">
+      <c r="D11" s="8" t="s">
         <v>133</v>
       </c>
+      <c r="E11" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
docs: documents 26/05/13_1 work
</commit_message>
<xml_diff>
--- a/doc/基本設計/00_勤怠管理システム_設計書.xlsx
+++ b/doc/基本設計/00_勤怠管理システム_設計書.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="TOP" sheetId="1" state="visible" r:id="rId3"/>
@@ -628,7 +628,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -679,6 +679,10 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -935,9 +939,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>674280</xdr:colOff>
+      <xdr:colOff>673920</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>10080</xdr:rowOff>
+      <xdr:rowOff>9720</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -947,7 +951,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="282960" y="1698840"/>
-          <a:ext cx="1524960" cy="577080"/>
+          <a:ext cx="1524600" cy="576720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1008,9 +1012,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>674280</xdr:colOff>
+      <xdr:colOff>673920</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>99360</xdr:rowOff>
+      <xdr:rowOff>99000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1020,7 +1024,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="282960" y="736560"/>
-          <a:ext cx="1524960" cy="577080"/>
+          <a:ext cx="1524600" cy="576720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1081,9 +1085,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>137160</xdr:colOff>
+      <xdr:colOff>136800</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>102960</xdr:rowOff>
+      <xdr:rowOff>102600</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1093,7 +1097,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2184120" y="2492640"/>
-          <a:ext cx="1524960" cy="577080"/>
+          <a:ext cx="1524600" cy="576720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1154,9 +1158,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>161280</xdr:colOff>
+      <xdr:colOff>160920</xdr:colOff>
       <xdr:row>29</xdr:row>
-      <xdr:rowOff>146520</xdr:rowOff>
+      <xdr:rowOff>146160</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1166,7 +1170,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2208240" y="4563000"/>
-          <a:ext cx="1524960" cy="577080"/>
+          <a:ext cx="1524600" cy="576720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1227,9 +1231,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>137160</xdr:colOff>
+      <xdr:colOff>136800</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>27360</xdr:rowOff>
+      <xdr:rowOff>27000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1239,7 +1243,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2184120" y="3456000"/>
-          <a:ext cx="1524960" cy="577080"/>
+          <a:ext cx="1524600" cy="576720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1300,9 +1304,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>172800</xdr:colOff>
+      <xdr:colOff>172440</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>13680</xdr:rowOff>
+      <xdr:rowOff>13320</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1312,7 +1316,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2219760" y="5580720"/>
-          <a:ext cx="1524960" cy="577080"/>
+          <a:ext cx="1524600" cy="576720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2087,7 +2091,7 @@
       <c r="E6" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="13" t="s">
         <v>68</v>
       </c>
       <c r="G6" s="8" t="s">
@@ -2206,7 +2210,7 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="14" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2306,7 +2310,7 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="14" t="s">
         <v>105</v>
       </c>
     </row>

</xml_diff>